<commit_message>
NBody benchmark, and some cosmetic improvments in other benchmarks
</commit_message>
<xml_diff>
--- a/docsrc/performance.xlsx
+++ b/docsrc/performance.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mueller/data/bau/docsrc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{246D0475-AB53-1140-9363-CA301284BF92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5501AD02-AC3A-8A41-A8C2-8121B33635ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4320" yWindow="500" windowWidth="34040" windowHeight="17500" activeTab="2" xr2:uid="{8BA8907E-A4D7-9D46-8614-8210467CB087}"/>
+    <workbookView xWindow="4320" yWindow="500" windowWidth="34040" windowHeight="17500" xr2:uid="{8BA8907E-A4D7-9D46-8614-8210467CB087}"/>
   </bookViews>
   <sheets>
     <sheet name="Performance" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="28">
   <si>
     <t>Benchmark</t>
   </si>
@@ -119,6 +119,9 @@
   </si>
   <si>
     <t>Stop-the-world GC pause in ms</t>
+  </si>
+  <si>
+    <t>Nbody</t>
   </si>
 </sst>
 </file>
@@ -817,6 +820,113 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000004-9C4A-2A4F-8C3D-1F740C03D694}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="5"/>
+          <c:order val="5"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Performance!$B$10</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Nbody</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent6"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>Performance!$C$4:$L$4</c:f>
+              <c:strCache>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>Bau</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>C</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Go</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Java</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Nim</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>PyPy</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Rust</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Swift</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Vlang</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Zig</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Performance!$C$10:$L$10</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>1.5</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1.4</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1.5</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1.9</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1.6</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>10.4</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1.7</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1.7</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1.6</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1.5</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-C3FE-7147-B843-EA0864A67C7F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1151,16 +1261,16 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>222</c:v>
+                  <c:v>354</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>5410</c:v>
+                  <c:v>9349</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2086</c:v>
+                  <c:v>3496</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2595</c:v>
+                  <c:v>4572</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1222,16 +1332,16 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>227</c:v>
+                  <c:v>354</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>5396</c:v>
+                  <c:v>9324</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2063</c:v>
+                  <c:v>3506</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2698</c:v>
+                  <c:v>4668</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1293,16 +1403,16 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>252</c:v>
+                  <c:v>381</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>6096</c:v>
+                  <c:v>10311</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2351</c:v>
+                  <c:v>3808</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>3068</c:v>
+                  <c:v>5252</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1364,16 +1474,16 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>283</c:v>
+                  <c:v>433</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>6571</c:v>
+                  <c:v>10997</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2542</c:v>
+                  <c:v>4114</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>3195</c:v>
+                  <c:v>5416</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1435,16 +1545,16 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>306</c:v>
+                  <c:v>456</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>6726</c:v>
+                  <c:v>10800</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2734</c:v>
+                  <c:v>4259</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>3028</c:v>
+                  <c:v>4993</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1506,16 +1616,16 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>277</c:v>
+                  <c:v>436</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>6953</c:v>
+                  <c:v>11901</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2590</c:v>
+                  <c:v>4717</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>3501</c:v>
+                  <c:v>5676</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1579,16 +1689,16 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>334</c:v>
+                  <c:v>483</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>7037</c:v>
+                  <c:v>11208</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2764</c:v>
+                  <c:v>4306</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>3217</c:v>
+                  <c:v>5230</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1652,16 +1762,16 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>306</c:v>
+                  <c:v>455</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>7268</c:v>
+                  <c:v>11821</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2604</c:v>
+                  <c:v>4186</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>3477</c:v>
+                  <c:v>5709</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1725,16 +1835,16 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>278</c:v>
+                  <c:v>430</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>7928</c:v>
+                  <c:v>13126</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>3322</c:v>
+                  <c:v>5449</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>3601</c:v>
+                  <c:v>5960</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1798,16 +1908,16 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>340</c:v>
+                  <c:v>491</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>8314</c:v>
+                  <c:v>12778</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>3311</c:v>
+                  <c:v>4885</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>3693</c:v>
+                  <c:v>5854</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1871,16 +1981,16 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>376</c:v>
+                  <c:v>538</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>10209</c:v>
+                  <c:v>15363</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>3526</c:v>
+                  <c:v>5306</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5011</c:v>
+                  <c:v>7495</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2258,34 +2368,34 @@
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.0225225225225225</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.1351351351351351</c:v>
+                  <c:v>1.076271186440678</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1.2747747747747749</c:v>
+                  <c:v>1.2231638418079096</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1.3783783783783783</c:v>
+                  <c:v>1.2881355932203389</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1.2477477477477477</c:v>
+                  <c:v>1.231638418079096</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1.5045045045045045</c:v>
+                  <c:v>1.3644067796610169</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1.3783783783783783</c:v>
+                  <c:v>1.2853107344632768</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1.2522522522522523</c:v>
+                  <c:v>1.2146892655367232</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>1.5315315315315314</c:v>
+                  <c:v>1.3870056497175141</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1.6936936936936937</c:v>
+                  <c:v>1.5197740112994351</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2371,34 +2481,34 @@
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.99741219963031424</c:v>
+                  <c:v>0.99732591721039687</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.1268022181146025</c:v>
+                  <c:v>1.1028987057439299</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1.2146025878003697</c:v>
+                  <c:v>1.1762755374906408</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1.2432532347504621</c:v>
+                  <c:v>1.1552037651085678</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1.2852125693160812</c:v>
+                  <c:v>1.2729703711626912</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1.3007393715341959</c:v>
+                  <c:v>1.1988447962348916</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1.3434380776340111</c:v>
+                  <c:v>1.264413306235961</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1.4654343807763401</c:v>
+                  <c:v>1.4040004278532463</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>1.5367837338262476</c:v>
+                  <c:v>1.3667771954219703</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1.8870609981515711</c:v>
+                  <c:v>1.6432773558669378</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2484,34 +2594,34 @@
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.98897411313518691</c:v>
+                  <c:v>1.0028604118993134</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.1270373921380632</c:v>
+                  <c:v>1.0892448512585813</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1.2186001917545541</c:v>
+                  <c:v>1.1767734553775744</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1.3106423777564717</c:v>
+                  <c:v>1.2182494279176201</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1.2416107382550334</c:v>
+                  <c:v>1.3492562929061784</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1.3250239693192714</c:v>
+                  <c:v>1.2316933638443937</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1.2483221476510067</c:v>
+                  <c:v>1.1973684210526316</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1.592521572387344</c:v>
+                  <c:v>1.5586384439359269</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>1.587248322147651</c:v>
+                  <c:v>1.3973112128146452</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1.6903163950143816</c:v>
+                  <c:v>1.5177345537757436</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2597,34 +2707,34 @@
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.0396917148362235</c:v>
+                  <c:v>1.0209973753280841</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.1822736030828516</c:v>
+                  <c:v>1.1487314085739282</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1.23121387283237</c:v>
+                  <c:v>1.1846019247594051</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1.166859344894027</c:v>
+                  <c:v>1.0920822397200349</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1.3491329479768785</c:v>
+                  <c:v>1.2414698162729658</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1.2396917148362234</c:v>
+                  <c:v>1.1439195100612425</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1.3398843930635838</c:v>
+                  <c:v>1.2486876640419948</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1.3876685934489403</c:v>
+                  <c:v>1.3035870516185477</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>1.4231213872832371</c:v>
+                  <c:v>1.2804024496937882</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1.9310211946050098</c:v>
+                  <c:v>1.639326334208224</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2707,37 +2817,37 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="11"/>
                 <c:pt idx="0">
-                  <c:v>1</c:v>
+                  <c:v>0.99999999999999989</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.93519882179675995</c:v>
+                  <c:v>0.93305439330543927</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.99263622974963184</c:v>
+                  <c:v>1.0150627615062762</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1.2268041237113403</c:v>
+                  <c:v>1.1983263598326359</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1.3019145802650958</c:v>
+                  <c:v>1.1983263598326359</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1.2739322533136965</c:v>
+                  <c:v>1.2359832635983263</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1.5022091310751104</c:v>
+                  <c:v>1.3615062761506276</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1.6583210603829159</c:v>
+                  <c:v>1.5313807531380752</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1.4830633284241532</c:v>
+                  <c:v>1.4100418410041839</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>1.8335787923416789</c:v>
+                  <c:v>1.6200836820083682</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>2.4491899852724592</c:v>
+                  <c:v>2.1037656903765689</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5539,13 +5649,13 @@
     <xdr:from>
       <xdr:col>9</xdr:col>
       <xdr:colOff>59947</xdr:colOff>
-      <xdr:row>13</xdr:row>
+      <xdr:row>14</xdr:row>
       <xdr:rowOff>6846</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>245270</xdr:colOff>
-      <xdr:row>13</xdr:row>
+      <xdr:row>14</xdr:row>
       <xdr:rowOff>235229</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -5605,13 +5715,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>171621</xdr:colOff>
-      <xdr:row>10</xdr:row>
+      <xdr:row>11</xdr:row>
       <xdr:rowOff>96109</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
       <xdr:colOff>36727</xdr:colOff>
-      <xdr:row>23</xdr:row>
+      <xdr:row>24</xdr:row>
       <xdr:rowOff>203372</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -5641,13 +5751,13 @@
     <xdr:from>
       <xdr:col>9</xdr:col>
       <xdr:colOff>77229</xdr:colOff>
-      <xdr:row>13</xdr:row>
+      <xdr:row>14</xdr:row>
       <xdr:rowOff>137298</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>231690</xdr:colOff>
-      <xdr:row>14</xdr:row>
+      <xdr:row>15</xdr:row>
       <xdr:rowOff>42905</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
@@ -5691,13 +5801,13 @@
     <xdr:from>
       <xdr:col>9</xdr:col>
       <xdr:colOff>66588</xdr:colOff>
-      <xdr:row>13</xdr:row>
+      <xdr:row>14</xdr:row>
       <xdr:rowOff>15104</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>221049</xdr:colOff>
-      <xdr:row>13</xdr:row>
+      <xdr:row>14</xdr:row>
       <xdr:rowOff>186725</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
@@ -6175,7 +6285,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{430266A2-5A9C-AA42-B61E-0693631C31C7}">
-  <dimension ref="B4:O23"/>
+  <dimension ref="B4:O24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="25.83203125" bestFit="1" customWidth="1"/>
@@ -6261,7 +6371,7 @@
         <v>67</v>
       </c>
       <c r="O5">
-        <f t="shared" ref="O5:O10" si="0">N5/H5</f>
+        <f t="shared" ref="O5:O11" si="0">N5/H5</f>
         <v>12.181818181818182</v>
       </c>
     </row>
@@ -6434,73 +6544,106 @@
       </c>
     </row>
     <row r="10" spans="2:15" ht="21" x14ac:dyDescent="0.25">
-      <c r="B10" s="1"/>
+      <c r="B10" s="1" t="s">
+        <v>27</v>
+      </c>
       <c r="C10" s="1">
-        <f t="shared" ref="C10:I10" si="1">SUM(C5:C9)</f>
-        <v>9.3000000000000007</v>
+        <v>1.5</v>
       </c>
       <c r="D10" s="1">
-        <f t="shared" si="1"/>
-        <v>8.2000000000000011</v>
+        <v>1.4</v>
       </c>
       <c r="E10" s="1">
-        <f t="shared" si="1"/>
-        <v>12.5</v>
+        <v>1.5</v>
       </c>
       <c r="F10" s="1">
-        <f t="shared" si="1"/>
-        <v>10.5</v>
+        <v>1.9</v>
       </c>
       <c r="G10" s="1">
-        <f t="shared" si="1"/>
-        <v>33</v>
+        <v>1.6</v>
       </c>
       <c r="H10" s="1">
-        <f t="shared" si="1"/>
-        <v>30.599999999999998</v>
+        <v>10.4</v>
       </c>
       <c r="I10" s="1">
-        <f t="shared" si="1"/>
-        <v>9.6999999999999993</v>
+        <v>1.7</v>
       </c>
       <c r="J10" s="1">
-        <f t="shared" ref="J10" si="2">SUM(J5:J9)</f>
-        <v>28.7</v>
+        <v>1.7</v>
       </c>
       <c r="K10" s="1">
-        <f t="shared" ref="K10" si="3">SUM(K5:K9)</f>
-        <v>12.3</v>
+        <v>1.6</v>
       </c>
       <c r="L10" s="1">
-        <f t="shared" ref="L10:N10" si="4">SUM(L5:L9)</f>
-        <v>19.8</v>
+        <v>1.5</v>
       </c>
       <c r="N10" s="1">
-        <f t="shared" si="4"/>
-        <v>392.8</v>
+        <v>167</v>
       </c>
       <c r="O10">
         <f t="shared" si="0"/>
-        <v>12.836601307189543</v>
-      </c>
-    </row>
-    <row r="12" spans="2:15" ht="21" x14ac:dyDescent="0.25">
-      <c r="B12" s="1"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
-      <c r="G12" s="2"/>
-      <c r="H12" s="2"/>
+        <v>16.057692307692307</v>
+      </c>
+    </row>
+    <row r="11" spans="2:15" ht="21" x14ac:dyDescent="0.25">
+      <c r="B11" s="1"/>
+      <c r="C11" s="1">
+        <f t="shared" ref="C11:L11" si="1">SUM(C5:C10)</f>
+        <v>10.8</v>
+      </c>
+      <c r="D11" s="1">
+        <f t="shared" si="1"/>
+        <v>9.6000000000000014</v>
+      </c>
+      <c r="E11" s="1">
+        <f t="shared" si="1"/>
+        <v>14</v>
+      </c>
+      <c r="F11" s="1">
+        <f t="shared" si="1"/>
+        <v>12.4</v>
+      </c>
+      <c r="G11" s="1">
+        <f t="shared" si="1"/>
+        <v>34.6</v>
+      </c>
+      <c r="H11" s="1">
+        <f t="shared" si="1"/>
+        <v>41</v>
+      </c>
+      <c r="I11" s="1">
+        <f t="shared" si="1"/>
+        <v>11.399999999999999</v>
+      </c>
+      <c r="J11" s="1">
+        <f t="shared" si="1"/>
+        <v>30.4</v>
+      </c>
+      <c r="K11" s="1">
+        <f t="shared" si="1"/>
+        <v>13.9</v>
+      </c>
+      <c r="L11" s="1">
+        <f t="shared" si="1"/>
+        <v>21.3</v>
+      </c>
+      <c r="N11" s="1">
+        <f>SUM(N5:N10)</f>
+        <v>559.79999999999995</v>
+      </c>
+      <c r="O11">
+        <f t="shared" si="0"/>
+        <v>13.653658536585365</v>
+      </c>
     </row>
     <row r="13" spans="2:15" ht="21" x14ac:dyDescent="0.25">
       <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
-      <c r="F13" s="1"/>
-      <c r="G13" s="1"/>
-      <c r="H13" s="1"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+      <c r="G13" s="2"/>
+      <c r="H13" s="2"/>
     </row>
     <row r="14" spans="2:15" ht="21" x14ac:dyDescent="0.25">
       <c r="B14" s="1"/>
@@ -6537,52 +6680,61 @@
       <c r="F17" s="1"/>
       <c r="G17" s="1"/>
       <c r="H17" s="1"/>
-      <c r="K17" s="5">
+    </row>
+    <row r="18" spans="2:14" ht="21" x14ac:dyDescent="0.25">
+      <c r="B18" s="1"/>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
+      <c r="F18" s="1"/>
+      <c r="G18" s="1"/>
+      <c r="H18" s="1"/>
+      <c r="K18" s="5">
         <v>0.42202546296296295</v>
       </c>
     </row>
-    <row r="18" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="K18" s="5">
+    <row r="19" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="K19" s="5">
         <v>0.4258912037037037</v>
       </c>
-      <c r="L18" s="5">
-        <f>K18-K17</f>
+      <c r="L19" s="5">
+        <f>K19-K18</f>
         <v>3.8657407407407529E-3</v>
       </c>
-      <c r="M18">
+      <c r="M19">
         <v>40</v>
       </c>
     </row>
-    <row r="19" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="M19">
+    <row r="20" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="M20">
         <f>60*5+30</f>
         <v>330</v>
       </c>
-      <c r="N19">
-        <f>M19/40</f>
+      <c r="N20">
+        <f>M20/40</f>
         <v>8.25</v>
       </c>
     </row>
-    <row r="20" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="N20" t="s">
+    <row r="21" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="N21" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="21" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="N21">
+    <row r="22" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="N22">
         <f>8.25 * 2000</f>
         <v>16500</v>
-      </c>
-    </row>
-    <row r="22" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="N22">
-        <f>N21/60</f>
-        <v>275</v>
       </c>
     </row>
     <row r="23" spans="2:14" x14ac:dyDescent="0.2">
       <c r="N23">
         <f>N22/60</f>
+        <v>275</v>
+      </c>
+    </row>
+    <row r="24" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="N24">
+        <f>N23/60</f>
         <v>4.583333333333333</v>
       </c>
     </row>
@@ -6646,22 +6798,22 @@
         <v>11</v>
       </c>
       <c r="C3">
-        <v>222</v>
+        <v>354</v>
       </c>
       <c r="D3">
-        <v>5410</v>
+        <v>9349</v>
       </c>
       <c r="E3">
-        <v>2086</v>
+        <v>3496</v>
       </c>
       <c r="F3">
-        <v>2595</v>
+        <v>4572</v>
       </c>
       <c r="G3">
-        <v>679</v>
+        <v>1195</v>
       </c>
       <c r="H3">
-        <v>50</v>
+        <v>87</v>
       </c>
       <c r="I3" s="4" t="str">
         <f>B3</f>
@@ -6685,7 +6837,7 @@
       </c>
       <c r="N3">
         <f t="shared" ref="N3" si="3">1/G$3*G3</f>
-        <v>1</v>
+        <v>0.99999999999999989</v>
       </c>
     </row>
     <row r="4" spans="2:21" x14ac:dyDescent="0.2">
@@ -6693,22 +6845,22 @@
         <v>1</v>
       </c>
       <c r="C4">
-        <v>227</v>
+        <v>354</v>
       </c>
       <c r="D4">
-        <v>5396</v>
+        <v>9324</v>
       </c>
       <c r="E4">
-        <v>2063</v>
+        <v>3506</v>
       </c>
       <c r="F4">
-        <v>2698</v>
+        <v>4668</v>
       </c>
       <c r="G4">
-        <v>635</v>
+        <v>1115</v>
       </c>
       <c r="H4">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="I4" s="4" t="str">
         <f t="shared" ref="I4:I12" si="4">B4</f>
@@ -6716,47 +6868,47 @@
       </c>
       <c r="J4">
         <f t="shared" ref="J4:J12" si="5">1/C$3*C4</f>
-        <v>1.0225225225225225</v>
+        <v>1</v>
       </c>
       <c r="K4">
         <f t="shared" ref="K4:K12" si="6">1/D$3*D4</f>
-        <v>0.99741219963031424</v>
+        <v>0.99732591721039687</v>
       </c>
       <c r="L4">
         <f t="shared" ref="L4:L12" si="7">1/E$3*E4</f>
-        <v>0.98897411313518691</v>
+        <v>1.0028604118993134</v>
       </c>
       <c r="M4">
         <f t="shared" ref="M4:M12" si="8">1/F$3*F4</f>
-        <v>1.0396917148362235</v>
+        <v>1.0209973753280841</v>
       </c>
       <c r="N4">
         <f t="shared" ref="N4:N12" si="9">1/G$3*G4</f>
-        <v>0.93519882179675995</v>
+        <v>0.93305439330543927</v>
       </c>
       <c r="P4">
         <f>J4-J$3</f>
-        <v>2.2522522522522515E-2</v>
+        <v>0</v>
       </c>
       <c r="Q4">
         <f t="shared" ref="Q4:Q12" si="10">K4-K$3</f>
-        <v>-2.5878003696857554E-3</v>
+        <v>-2.6740827896031272E-3</v>
       </c>
       <c r="R4">
         <f t="shared" ref="R4:R12" si="11">L4-L$3</f>
-        <v>-1.1025886864813095E-2</v>
+        <v>2.8604118993134087E-3</v>
       </c>
       <c r="S4">
         <f t="shared" ref="S4:S12" si="12">M4-M$3</f>
-        <v>3.9691714836223468E-2</v>
+        <v>2.09973753280841E-2</v>
       </c>
       <c r="T4">
         <f t="shared" ref="T4:T12" si="13">N4-N$3</f>
-        <v>-6.4801178203240051E-2</v>
+        <v>-6.6945606694560622E-2</v>
       </c>
       <c r="U4">
         <f>SUM(P4:T4)</f>
-        <v>-1.6200628078992918E-2</v>
+        <v>-4.576190225676624E-2</v>
       </c>
     </row>
     <row r="5" spans="2:21" x14ac:dyDescent="0.2">
@@ -6764,22 +6916,22 @@
         <v>23</v>
       </c>
       <c r="C5">
-        <v>252</v>
+        <v>381</v>
       </c>
       <c r="D5">
-        <v>6096</v>
+        <v>10311</v>
       </c>
       <c r="E5">
-        <v>2351</v>
+        <v>3808</v>
       </c>
       <c r="F5">
-        <v>3068</v>
+        <v>5252</v>
       </c>
       <c r="G5">
-        <v>674</v>
+        <v>1213</v>
       </c>
       <c r="H5">
-        <v>4</v>
+        <v>39</v>
       </c>
       <c r="I5" s="4" t="str">
         <f t="shared" si="4"/>
@@ -6787,47 +6939,47 @@
       </c>
       <c r="J5">
         <f t="shared" si="5"/>
-        <v>1.1351351351351351</v>
+        <v>1.076271186440678</v>
       </c>
       <c r="K5">
         <f t="shared" si="6"/>
-        <v>1.1268022181146025</v>
+        <v>1.1028987057439299</v>
       </c>
       <c r="L5">
         <f t="shared" si="7"/>
-        <v>1.1270373921380632</v>
+        <v>1.0892448512585813</v>
       </c>
       <c r="M5">
         <f t="shared" si="8"/>
-        <v>1.1822736030828516</v>
+        <v>1.1487314085739282</v>
       </c>
       <c r="N5">
         <f t="shared" si="9"/>
-        <v>0.99263622974963184</v>
+        <v>1.0150627615062762</v>
       </c>
       <c r="P5">
         <f t="shared" ref="P5:P12" si="14">J5-J$3</f>
-        <v>0.13513513513513509</v>
+        <v>7.6271186440677985E-2</v>
       </c>
       <c r="Q5">
         <f t="shared" si="10"/>
-        <v>0.12680221811460246</v>
+        <v>0.1028987057439299</v>
       </c>
       <c r="R5">
         <f t="shared" si="11"/>
-        <v>0.1270373921380632</v>
+        <v>8.9244851258581281E-2</v>
       </c>
       <c r="S5">
         <f t="shared" si="12"/>
-        <v>0.18227360308285157</v>
+        <v>0.14873140857392819</v>
       </c>
       <c r="T5">
         <f t="shared" si="13"/>
-        <v>-7.3637702503681624E-3</v>
+        <v>1.5062761506276279E-2</v>
       </c>
       <c r="U5">
         <f t="shared" ref="U5:U12" si="15">SUM(P5:T5)</f>
-        <v>0.56388457822028415</v>
+        <v>0.43220891352339363</v>
       </c>
     </row>
     <row r="6" spans="2:21" x14ac:dyDescent="0.2">
@@ -6835,22 +6987,22 @@
         <v>20</v>
       </c>
       <c r="C6">
-        <v>283</v>
+        <v>433</v>
       </c>
       <c r="D6">
-        <v>6571</v>
+        <v>10997</v>
       </c>
       <c r="E6">
-        <v>2542</v>
+        <v>4114</v>
       </c>
       <c r="F6">
-        <v>3195</v>
+        <v>5416</v>
       </c>
       <c r="G6">
-        <v>833</v>
+        <v>1432</v>
       </c>
       <c r="H6">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="I6" s="4" t="str">
         <f t="shared" si="4"/>
@@ -6858,47 +7010,47 @@
       </c>
       <c r="J6">
         <f t="shared" si="5"/>
-        <v>1.2747747747747749</v>
+        <v>1.2231638418079096</v>
       </c>
       <c r="K6">
         <f t="shared" si="6"/>
-        <v>1.2146025878003697</v>
+        <v>1.1762755374906408</v>
       </c>
       <c r="L6">
         <f t="shared" si="7"/>
-        <v>1.2186001917545541</v>
+        <v>1.1767734553775744</v>
       </c>
       <c r="M6">
         <f t="shared" si="8"/>
-        <v>1.23121387283237</v>
+        <v>1.1846019247594051</v>
       </c>
       <c r="N6">
         <f t="shared" si="9"/>
-        <v>1.2268041237113403</v>
+        <v>1.1983263598326359</v>
       </c>
       <c r="P6">
         <f t="shared" si="14"/>
-        <v>0.27477477477477485</v>
+        <v>0.2231638418079096</v>
       </c>
       <c r="Q6">
         <f t="shared" si="10"/>
-        <v>0.21460258780036967</v>
+        <v>0.17627553749064084</v>
       </c>
       <c r="R6">
         <f t="shared" si="11"/>
-        <v>0.21860019175455414</v>
+        <v>0.17677345537757438</v>
       </c>
       <c r="S6">
         <f t="shared" si="12"/>
-        <v>0.23121387283237005</v>
+        <v>0.18460192475940507</v>
       </c>
       <c r="T6">
         <f t="shared" si="13"/>
-        <v>0.22680412371134029</v>
+        <v>0.19832635983263602</v>
       </c>
       <c r="U6">
         <f t="shared" si="15"/>
-        <v>1.165995550873409</v>
+        <v>0.95914111926816592</v>
       </c>
     </row>
     <row r="7" spans="2:21" x14ac:dyDescent="0.2">
@@ -6906,22 +7058,22 @@
         <v>24</v>
       </c>
       <c r="C7">
-        <v>306</v>
+        <v>456</v>
       </c>
       <c r="D7">
-        <v>6726</v>
+        <v>10800</v>
       </c>
       <c r="E7">
-        <v>2734</v>
+        <v>4259</v>
       </c>
       <c r="F7">
-        <v>3028</v>
+        <v>4993</v>
       </c>
       <c r="G7">
-        <v>884</v>
+        <v>1432</v>
       </c>
       <c r="H7">
-        <v>81</v>
+        <v>118</v>
       </c>
       <c r="I7" s="4" t="str">
         <f t="shared" si="4"/>
@@ -6929,47 +7081,47 @@
       </c>
       <c r="J7">
         <f t="shared" si="5"/>
-        <v>1.3783783783783783</v>
+        <v>1.2881355932203389</v>
       </c>
       <c r="K7">
         <f t="shared" si="6"/>
-        <v>1.2432532347504621</v>
+        <v>1.1552037651085678</v>
       </c>
       <c r="L7">
         <f t="shared" si="7"/>
-        <v>1.3106423777564717</v>
+        <v>1.2182494279176201</v>
       </c>
       <c r="M7">
         <f t="shared" si="8"/>
-        <v>1.166859344894027</v>
+        <v>1.0920822397200349</v>
       </c>
       <c r="N7">
         <f t="shared" si="9"/>
-        <v>1.3019145802650958</v>
+        <v>1.1983263598326359</v>
       </c>
       <c r="P7">
         <f t="shared" si="14"/>
-        <v>0.37837837837837829</v>
+        <v>0.28813559322033888</v>
       </c>
       <c r="Q7">
         <f t="shared" si="10"/>
-        <v>0.24325323475046212</v>
+        <v>0.15520376510856781</v>
       </c>
       <c r="R7">
         <f t="shared" si="11"/>
-        <v>0.31064237775647174</v>
+        <v>0.21824942791762014</v>
       </c>
       <c r="S7">
         <f t="shared" si="12"/>
-        <v>0.16685934489402698</v>
+        <v>9.2082239720034931E-2</v>
       </c>
       <c r="T7">
         <f t="shared" si="13"/>
-        <v>0.30191458026509577</v>
+        <v>0.19832635983263602</v>
       </c>
       <c r="U7">
         <f t="shared" si="15"/>
-        <v>1.4010479160444349</v>
+        <v>0.95199738579919779</v>
       </c>
     </row>
     <row r="8" spans="2:21" x14ac:dyDescent="0.2">
@@ -6977,22 +7129,22 @@
         <v>19</v>
       </c>
       <c r="C8">
-        <v>277</v>
+        <v>436</v>
       </c>
       <c r="D8">
-        <v>6953</v>
+        <v>11901</v>
       </c>
       <c r="E8">
-        <v>2590</v>
+        <v>4717</v>
       </c>
       <c r="F8">
-        <v>3501</v>
+        <v>5676</v>
       </c>
       <c r="G8">
-        <v>865</v>
+        <v>1477</v>
       </c>
       <c r="H8">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="I8" s="4" t="str">
         <f t="shared" si="4"/>
@@ -7000,47 +7152,47 @@
       </c>
       <c r="J8">
         <f t="shared" si="5"/>
-        <v>1.2477477477477477</v>
+        <v>1.231638418079096</v>
       </c>
       <c r="K8">
         <f t="shared" si="6"/>
-        <v>1.2852125693160812</v>
+        <v>1.2729703711626912</v>
       </c>
       <c r="L8">
         <f t="shared" si="7"/>
-        <v>1.2416107382550334</v>
+        <v>1.3492562929061784</v>
       </c>
       <c r="M8">
         <f t="shared" si="8"/>
-        <v>1.3491329479768785</v>
+        <v>1.2414698162729658</v>
       </c>
       <c r="N8">
         <f t="shared" si="9"/>
-        <v>1.2739322533136965</v>
+        <v>1.2359832635983263</v>
       </c>
       <c r="P8">
         <f t="shared" si="14"/>
-        <v>0.24774774774774766</v>
+        <v>0.23163841807909602</v>
       </c>
       <c r="Q8">
         <f t="shared" si="10"/>
-        <v>0.28521256931608119</v>
+        <v>0.27297037116269118</v>
       </c>
       <c r="R8">
         <f t="shared" si="11"/>
-        <v>0.24161073825503343</v>
+        <v>0.34925629290617843</v>
       </c>
       <c r="S8">
         <f t="shared" si="12"/>
-        <v>0.34913294797687855</v>
+        <v>0.24146981627296582</v>
       </c>
       <c r="T8">
         <f t="shared" si="13"/>
-        <v>0.27393225331369653</v>
+        <v>0.23598326359832644</v>
       </c>
       <c r="U8">
         <f t="shared" si="15"/>
-        <v>1.3976362566094374</v>
+        <v>1.331318162019258</v>
       </c>
     </row>
     <row r="9" spans="2:21" x14ac:dyDescent="0.2">
@@ -7048,22 +7200,22 @@
         <v>3</v>
       </c>
       <c r="C9">
-        <v>334</v>
+        <v>483</v>
       </c>
       <c r="D9" s="3">
-        <v>7037</v>
+        <v>11208</v>
       </c>
       <c r="E9">
-        <v>2764</v>
+        <v>4306</v>
       </c>
       <c r="F9">
-        <v>3217</v>
+        <v>5230</v>
       </c>
       <c r="G9">
-        <v>1020</v>
+        <v>1627</v>
       </c>
       <c r="H9">
-        <v>9</v>
+        <v>44</v>
       </c>
       <c r="I9" s="4" t="str">
         <f t="shared" si="4"/>
@@ -7071,47 +7223,47 @@
       </c>
       <c r="J9">
         <f t="shared" si="5"/>
-        <v>1.5045045045045045</v>
+        <v>1.3644067796610169</v>
       </c>
       <c r="K9">
         <f t="shared" si="6"/>
-        <v>1.3007393715341959</v>
+        <v>1.1988447962348916</v>
       </c>
       <c r="L9">
         <f t="shared" si="7"/>
-        <v>1.3250239693192714</v>
+        <v>1.2316933638443937</v>
       </c>
       <c r="M9">
         <f t="shared" si="8"/>
-        <v>1.2396917148362234</v>
+        <v>1.1439195100612425</v>
       </c>
       <c r="N9">
         <f t="shared" si="9"/>
-        <v>1.5022091310751104</v>
+        <v>1.3615062761506276</v>
       </c>
       <c r="P9">
         <f t="shared" si="14"/>
-        <v>0.50450450450450446</v>
+        <v>0.36440677966101687</v>
       </c>
       <c r="Q9">
         <f t="shared" si="10"/>
-        <v>0.30073937153419594</v>
+        <v>0.1988447962348916</v>
       </c>
       <c r="R9">
         <f t="shared" si="11"/>
-        <v>0.32502396931927136</v>
+        <v>0.23169336384439365</v>
       </c>
       <c r="S9">
         <f t="shared" si="12"/>
-        <v>0.23969171483622342</v>
+        <v>0.14391951006124248</v>
       </c>
       <c r="T9">
         <f t="shared" si="13"/>
-        <v>0.50220913107511045</v>
+        <v>0.36150627615062769</v>
       </c>
       <c r="U9">
         <f t="shared" si="15"/>
-        <v>1.8721686912693056</v>
+        <v>1.3003707259521722</v>
       </c>
     </row>
     <row r="10" spans="2:21" x14ac:dyDescent="0.2">
@@ -7119,22 +7271,22 @@
         <v>2</v>
       </c>
       <c r="C10">
-        <v>306</v>
+        <v>455</v>
       </c>
       <c r="D10" s="3">
-        <v>7268</v>
+        <v>11821</v>
       </c>
       <c r="E10">
-        <v>2604</v>
+        <v>4186</v>
       </c>
       <c r="F10">
-        <v>3477</v>
+        <v>5709</v>
       </c>
       <c r="G10">
-        <v>1126</v>
+        <v>1830</v>
       </c>
       <c r="H10">
-        <v>60</v>
+        <v>95</v>
       </c>
       <c r="I10" s="4" t="str">
         <f t="shared" si="4"/>
@@ -7142,47 +7294,47 @@
       </c>
       <c r="J10">
         <f t="shared" si="5"/>
-        <v>1.3783783783783783</v>
+        <v>1.2853107344632768</v>
       </c>
       <c r="K10">
         <f t="shared" si="6"/>
-        <v>1.3434380776340111</v>
+        <v>1.264413306235961</v>
       </c>
       <c r="L10">
         <f t="shared" si="7"/>
-        <v>1.2483221476510067</v>
+        <v>1.1973684210526316</v>
       </c>
       <c r="M10">
         <f t="shared" si="8"/>
-        <v>1.3398843930635838</v>
+        <v>1.2486876640419948</v>
       </c>
       <c r="N10">
         <f t="shared" si="9"/>
-        <v>1.6583210603829159</v>
+        <v>1.5313807531380752</v>
       </c>
       <c r="P10">
         <f t="shared" si="14"/>
-        <v>0.37837837837837829</v>
+        <v>0.28531073446327682</v>
       </c>
       <c r="Q10">
         <f t="shared" si="10"/>
-        <v>0.34343807763401113</v>
+        <v>0.26441330623596104</v>
       </c>
       <c r="R10">
         <f t="shared" si="11"/>
-        <v>0.24832214765100669</v>
+        <v>0.19736842105263164</v>
       </c>
       <c r="S10">
         <f t="shared" si="12"/>
-        <v>0.33988439306358376</v>
+        <v>0.24868766404199483</v>
       </c>
       <c r="T10">
         <f t="shared" si="13"/>
-        <v>0.65832106038291593</v>
+        <v>0.53138075313807531</v>
       </c>
       <c r="U10">
         <f t="shared" si="15"/>
-        <v>1.9683440571098958</v>
+        <v>1.5271608789319395</v>
       </c>
     </row>
     <row r="11" spans="2:21" x14ac:dyDescent="0.2">
@@ -7190,22 +7342,22 @@
         <v>4</v>
       </c>
       <c r="C11">
-        <v>278</v>
+        <v>430</v>
       </c>
       <c r="D11" s="3">
-        <v>7928</v>
+        <v>13126</v>
       </c>
       <c r="E11">
-        <v>3322</v>
+        <v>5449</v>
       </c>
       <c r="F11">
-        <v>3601</v>
+        <v>5960</v>
       </c>
       <c r="G11">
-        <v>1007</v>
+        <v>1685</v>
       </c>
       <c r="H11">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="I11" s="4" t="str">
         <f t="shared" si="4"/>
@@ -7213,47 +7365,47 @@
       </c>
       <c r="J11">
         <f t="shared" si="5"/>
-        <v>1.2522522522522523</v>
+        <v>1.2146892655367232</v>
       </c>
       <c r="K11">
         <f t="shared" si="6"/>
-        <v>1.4654343807763401</v>
+        <v>1.4040004278532463</v>
       </c>
       <c r="L11">
         <f t="shared" si="7"/>
-        <v>1.592521572387344</v>
+        <v>1.5586384439359269</v>
       </c>
       <c r="M11">
         <f t="shared" si="8"/>
-        <v>1.3876685934489403</v>
+        <v>1.3035870516185477</v>
       </c>
       <c r="N11">
         <f t="shared" si="9"/>
-        <v>1.4830633284241532</v>
+        <v>1.4100418410041839</v>
       </c>
       <c r="P11">
         <f t="shared" si="14"/>
-        <v>0.25225225225225234</v>
+        <v>0.21468926553672318</v>
       </c>
       <c r="Q11">
         <f t="shared" si="10"/>
-        <v>0.46543438077634014</v>
+        <v>0.4040004278532463</v>
       </c>
       <c r="R11">
         <f t="shared" si="11"/>
-        <v>0.59252157238734404</v>
+        <v>0.55863844393592688</v>
       </c>
       <c r="S11">
         <f t="shared" si="12"/>
-        <v>0.38766859344894034</v>
+        <v>0.30358705161854771</v>
       </c>
       <c r="T11">
         <f t="shared" si="13"/>
-        <v>0.48306332842415323</v>
+        <v>0.41004184100418406</v>
       </c>
       <c r="U11">
         <f t="shared" si="15"/>
-        <v>2.1809401272890301</v>
+        <v>1.8909570299486282</v>
       </c>
     </row>
     <row r="12" spans="2:21" x14ac:dyDescent="0.2">
@@ -7261,22 +7413,22 @@
         <v>5</v>
       </c>
       <c r="C12">
-        <v>340</v>
+        <v>491</v>
       </c>
       <c r="D12" s="3">
-        <v>8314</v>
+        <v>12778</v>
       </c>
       <c r="E12">
-        <v>3311</v>
+        <v>4885</v>
       </c>
       <c r="F12">
-        <v>3693</v>
+        <v>5854</v>
       </c>
       <c r="G12">
-        <v>1245</v>
+        <v>1936</v>
       </c>
       <c r="H12">
-        <v>65</v>
+        <v>103</v>
       </c>
       <c r="I12" s="4" t="str">
         <f t="shared" si="4"/>
@@ -7284,47 +7436,47 @@
       </c>
       <c r="J12">
         <f t="shared" si="5"/>
-        <v>1.5315315315315314</v>
+        <v>1.3870056497175141</v>
       </c>
       <c r="K12">
         <f t="shared" si="6"/>
-        <v>1.5367837338262476</v>
+        <v>1.3667771954219703</v>
       </c>
       <c r="L12">
         <f t="shared" si="7"/>
-        <v>1.587248322147651</v>
+        <v>1.3973112128146452</v>
       </c>
       <c r="M12">
         <f t="shared" si="8"/>
-        <v>1.4231213872832371</v>
+        <v>1.2804024496937882</v>
       </c>
       <c r="N12">
         <f t="shared" si="9"/>
-        <v>1.8335787923416789</v>
+        <v>1.6200836820083682</v>
       </c>
       <c r="P12">
         <f t="shared" si="14"/>
-        <v>0.53153153153153143</v>
+        <v>0.38700564971751406</v>
       </c>
       <c r="Q12">
         <f t="shared" si="10"/>
-        <v>0.53678373382624756</v>
+        <v>0.36677719542197029</v>
       </c>
       <c r="R12">
         <f t="shared" si="11"/>
-        <v>0.58724832214765099</v>
+        <v>0.39731121281464521</v>
       </c>
       <c r="S12">
         <f t="shared" si="12"/>
-        <v>0.42312138728323712</v>
+        <v>0.28040244969378825</v>
       </c>
       <c r="T12">
         <f t="shared" si="13"/>
-        <v>0.83357879234167886</v>
+        <v>0.62008368200836828</v>
       </c>
       <c r="U12">
         <f t="shared" si="15"/>
-        <v>2.9122637671303462</v>
+        <v>2.0515801896562862</v>
       </c>
     </row>
     <row r="13" spans="2:21" x14ac:dyDescent="0.2">
@@ -7332,22 +7484,22 @@
         <v>25</v>
       </c>
       <c r="C13">
-        <v>376</v>
+        <v>538</v>
       </c>
       <c r="D13" s="3">
-        <v>10209</v>
+        <v>15363</v>
       </c>
       <c r="E13">
-        <v>3526</v>
+        <v>5306</v>
       </c>
       <c r="F13">
-        <v>5011</v>
+        <v>7495</v>
       </c>
       <c r="G13">
-        <v>1663</v>
+        <v>2514</v>
       </c>
       <c r="H13">
-        <v>9</v>
+        <v>48</v>
       </c>
       <c r="I13" s="4" t="str">
         <f t="shared" ref="I13" si="16">B13</f>
@@ -7355,23 +7507,23 @@
       </c>
       <c r="J13">
         <f t="shared" ref="J13" si="17">1/C$3*C13</f>
-        <v>1.6936936936936937</v>
+        <v>1.5197740112994351</v>
       </c>
       <c r="K13">
         <f t="shared" ref="K13" si="18">1/D$3*D13</f>
-        <v>1.8870609981515711</v>
+        <v>1.6432773558669378</v>
       </c>
       <c r="L13">
         <f t="shared" ref="L13" si="19">1/E$3*E13</f>
-        <v>1.6903163950143816</v>
+        <v>1.5177345537757436</v>
       </c>
       <c r="M13">
         <f t="shared" ref="M13" si="20">1/F$3*F13</f>
-        <v>1.9310211946050098</v>
+        <v>1.639326334208224</v>
       </c>
       <c r="N13">
         <f t="shared" ref="N13" si="21">1/G$3*G13</f>
-        <v>2.4491899852724592</v>
+        <v>2.1037656903765689</v>
       </c>
     </row>
     <row r="14" spans="2:21" x14ac:dyDescent="0.2">

</xml_diff>